<commit_message>
Añadir vertical Precio y reclasificar reviews existentes
</commit_message>
<xml_diff>
--- a/holded_reviews.xlsx
+++ b/holded_reviews.xlsx
@@ -826,7 +826,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Precio</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Precio</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Precio</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">

</xml_diff>